<commit_message>
Change Unit Testing part
</commit_message>
<xml_diff>
--- a/template_files/Unit_Testing_Template.xlsx
+++ b/template_files/Unit_Testing_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\A- Main - LLM For Testing\Main Version\llms-for-testing-test\template_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C6A074-6344-468C-8F16-7F4BE9796FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447DB04C-AD31-4179-BCDE-C9529F18DFDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6EFD6933-DD0B-4386-8419-B2D064BD42A2}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{6EFD6933-DD0B-4386-8419-B2D064BD42A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,25 +34,34 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Test Case Type</t>
-  </si>
-  <si>
-    <t>Test Cases</t>
-  </si>
-  <si>
-    <t>&lt;Please Enter the Test Case Type
- here&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Please Enter the Test Cases here&gt;</t>
-  </si>
-  <si>
-    <t>Function Code</t>
-  </si>
-  <si>
-    <t>&lt;Please Enter the Function Code here&gt;</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t xml:space="preserve">Springboot Version
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input For a Function
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Function
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denpendent Codes
+</t>
+  </si>
+  <si>
+    <t>&lt;Enter the Denpendent Codes to here&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Please Enter the Function code here&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Enter the inputs for the function to here&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Enter the Springboot Version here&gt;</t>
   </si>
 </sst>
 </file>
@@ -130,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -142,6 +151,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -458,47 +470,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70713DFC-66D7-4EB6-9694-9CBA1164CD8E}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="38.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.5703125" customWidth="1"/>
+    <col min="2" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>2</v>
+    <row r="2" spans="1:5" s="1" customFormat="1" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3"/>
+      <c r="D2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>